<commit_message>
Fix issues where proposals were not being deleted and logged correctly
Implement proper handling for entry deletions in the change log, including UI updates, server-side logic for admin-only deletion, and improved error handling for delete operations and exports.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 0b66b356-8407-4786-a889-c9d2c96f6018
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/Gx2kXql
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-09.xlsx
+++ b/backups/proposal-log-2026-04-09.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="125">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -262,6 +262,9 @@
     <t>26-0208</t>
   </si>
   <si>
+    <t>Entertainment</t>
+  </si>
+  <si>
     <t>GT</t>
   </si>
   <si>
@@ -316,6 +319,9 @@
     <t>Nilda Puno</t>
   </si>
   <si>
+    <t>3000</t>
+  </si>
+  <si>
     <t>https://app.buildingconnected.com/opportunities/69c42fb71e34da5627943f29</t>
   </si>
   <si>
@@ -353,6 +359,9 @@
   </si>
   <si>
     <t>26-0217</t>
+  </si>
+  <si>
+    <t>KR</t>
   </si>
   <si>
     <t>https://app.buildingconnected.com/opportunities/69d3de61132a4642c558b4df</t>
@@ -1242,7 +1251,7 @@
         <v>16</v>
       </c>
       <c r="D11" t="s">
-        <v>17</v>
+        <v>83</v>
       </c>
       <c r="E11" t="s">
         <v>18</v>
@@ -1251,13 +1260,13 @@
         <v>19</v>
       </c>
       <c r="G11" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H11" t="s">
         <v>20</v>
       </c>
       <c r="I11" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J11" t="s">
         <v>58</v>
@@ -1277,13 +1286,13 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B12" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C12" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D12" t="s">
         <v>78</v>
@@ -1292,63 +1301,63 @@
         <v>18</v>
       </c>
       <c r="F12" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G12" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H12" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="I12" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="J12" t="s">
         <v>40</v>
       </c>
       <c r="K12" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="L12" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="M12" t="s">
         <v>17</v>
       </c>
       <c r="N12" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B13" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C13" t="s">
         <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E13" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F13" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G13" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H13" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="I13" t="s">
-        <v>57</v>
+        <v>102</v>
       </c>
       <c r="J13" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="K13" t="s">
         <v>17</v>
@@ -1360,33 +1369,33 @@
         <v>17</v>
       </c>
       <c r="N13" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B14" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="C14" t="s">
         <v>26</v>
       </c>
       <c r="D14" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="E14" t="s">
         <v>54</v>
       </c>
       <c r="F14" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="G14" t="s">
         <v>17</v>
       </c>
       <c r="H14" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="I14" t="s">
         <v>17</v>
@@ -1404,18 +1413,18 @@
         <v>17</v>
       </c>
       <c r="N14" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B15" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C15" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D15" t="s">
         <v>78</v>
@@ -1424,13 +1433,13 @@
         <v>37</v>
       </c>
       <c r="F15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G15" t="s">
         <v>17</v>
       </c>
       <c r="H15" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I15" t="s">
         <v>57</v>
@@ -1448,18 +1457,18 @@
         <v>17</v>
       </c>
       <c r="N15" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B16" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C16" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D16" t="s">
         <v>78</v>
@@ -1468,13 +1477,13 @@
         <v>37</v>
       </c>
       <c r="F16" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G16" t="s">
-        <v>17</v>
+        <v>116</v>
       </c>
       <c r="H16" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I16" t="s">
         <v>17</v>
@@ -1492,15 +1501,15 @@
         <v>17</v>
       </c>
       <c r="N16" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B17" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C17" t="s">
         <v>61</v>
@@ -1512,13 +1521,13 @@
         <v>27</v>
       </c>
       <c r="F17" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="G17" t="s">
         <v>17</v>
       </c>
       <c r="H17" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="I17" t="s">
         <v>17</v>
@@ -1536,18 +1545,18 @@
         <v>17</v>
       </c>
       <c r="N17" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B18" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C18" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D18" t="s">
         <v>78</v>
@@ -1556,13 +1565,13 @@
         <v>37</v>
       </c>
       <c r="F18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G18" t="s">
         <v>17</v>
       </c>
       <c r="H18" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I18" t="s">
         <v>17</v>
@@ -1580,7 +1589,7 @@
         <v>17</v>
       </c>
       <c r="N18" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enforce tool access permissions on the dashboard
Add feature keys to tools, integrate feature access checks into the HomePage component's render loop, and update permissions initialization to remove "submittal-builder" from default Estimator role features and existing Estimator user access.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: d3b943a8-a1ee-479f-a234-9aaff4b5af78
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/Hv7DBLR
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-09.xlsx
+++ b/backups/proposal-log-2026-04-09.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="119">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -193,157 +193,169 @@
     <t>https://app.buildingconnected.com/opportunities/69cfe3add7a6218079f9a6b3</t>
   </si>
   <si>
-    <t>26-0213</t>
+    <t>26-0212</t>
+  </si>
+  <si>
+    <t>Adidas Tanger Deer Park</t>
+  </si>
+  <si>
+    <t>LGA</t>
+  </si>
+  <si>
+    <t>2026-04-08</t>
+  </si>
+  <si>
+    <t>JW</t>
+  </si>
+  <si>
+    <t>Joseph Dinielli</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69cd0562786a720050b13b93</t>
+  </si>
+  <si>
+    <t>26-0211</t>
+  </si>
+  <si>
+    <t>Amazon SEA Legacy Space Refresh Medium GC Bid</t>
+  </si>
+  <si>
+    <t>2026-04-09</t>
+  </si>
+  <si>
+    <t>Merci Keathley</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69cc472c724d4f360623c300</t>
+  </si>
+  <si>
+    <t>26-0209</t>
+  </si>
+  <si>
+    <t>Flying Pickle Idaho Falls</t>
+  </si>
+  <si>
+    <t>GEG</t>
+  </si>
+  <si>
+    <t>Special Projects</t>
+  </si>
+  <si>
+    <t>2026-03-31</t>
+  </si>
+  <si>
+    <t>KR</t>
+  </si>
+  <si>
+    <t>Jake Marrujo</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69cc01834e68f2d35d122b59</t>
+  </si>
+  <si>
+    <t>26-0208</t>
+  </si>
+  <si>
+    <t>Entertainment</t>
+  </si>
+  <si>
+    <t>GT</t>
+  </si>
+  <si>
+    <t>10187</t>
+  </si>
+  <si>
+    <t>26-0207</t>
+  </si>
+  <si>
+    <t>Illumina Project SOL</t>
+  </si>
+  <si>
+    <t>SAN - SD</t>
+  </si>
+  <si>
+    <t>2026-04-21</t>
+  </si>
+  <si>
+    <t>HK</t>
+  </si>
+  <si>
+    <t>Vahid Balali</t>
+  </si>
+  <si>
+    <t>148686</t>
+  </si>
+  <si>
+    <t>2026-06-01</t>
+  </si>
+  <si>
+    <t>2026-11-01</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c6e1d59317e8e48f1c9603</t>
+  </si>
+  <si>
+    <t>26-0206</t>
+  </si>
+  <si>
+    <t>Inglewood Transit Connector RFQ</t>
+  </si>
+  <si>
+    <t>Retail</t>
+  </si>
+  <si>
+    <t>2026-03-25</t>
+  </si>
+  <si>
+    <t>2026-04-11</t>
+  </si>
+  <si>
+    <t>Nilda Puno</t>
+  </si>
+  <si>
+    <t>3000</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69c42fb71e34da5627943f29</t>
+  </si>
+  <si>
+    <t>26-0215</t>
+  </si>
+  <si>
+    <t>33P Affordable Housing Multi-Family Devlopment</t>
+  </si>
+  <si>
+    <t>Residential</t>
+  </si>
+  <si>
+    <t>2026-04-15</t>
+  </si>
+  <si>
+    <t>Jon Smith</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69d046a028ff4e0032ca893c</t>
+  </si>
+  <si>
+    <t>26-0219</t>
+  </si>
+  <si>
+    <t>Station 33 Bldg 4 Food Hall SD Budget</t>
   </si>
   <si>
     <t>DFW</t>
   </si>
   <si>
-    <t>Christman Weeks</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69ce6ad9ffa00f5f6b96a4d9</t>
-  </si>
-  <si>
-    <t>26-0212</t>
-  </si>
-  <si>
-    <t>Adidas Tanger Deer Park</t>
-  </si>
-  <si>
-    <t>LGA</t>
-  </si>
-  <si>
-    <t>2026-04-08</t>
-  </si>
-  <si>
-    <t>Joseph Dinielli</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69cd0562786a720050b13b93</t>
-  </si>
-  <si>
-    <t>26-0211</t>
-  </si>
-  <si>
-    <t>Amazon SEA Legacy Space Refresh Medium GC Bid</t>
-  </si>
-  <si>
-    <t>2026-04-09</t>
-  </si>
-  <si>
-    <t>Merci Keathley</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69cc472c724d4f360623c300</t>
-  </si>
-  <si>
-    <t>26-0209</t>
-  </si>
-  <si>
-    <t>Flying Pickle Idaho Falls</t>
-  </si>
-  <si>
-    <t>GEG</t>
-  </si>
-  <si>
-    <t>Special Projects</t>
-  </si>
-  <si>
-    <t>2026-03-31</t>
-  </si>
-  <si>
-    <t>Jake Marrujo</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69cc01834e68f2d35d122b59</t>
-  </si>
-  <si>
-    <t>26-0208</t>
-  </si>
-  <si>
-    <t>Entertainment</t>
-  </si>
-  <si>
-    <t>GT</t>
-  </si>
-  <si>
-    <t>10187</t>
-  </si>
-  <si>
-    <t>26-0207</t>
-  </si>
-  <si>
-    <t>Illumina Project SOL</t>
-  </si>
-  <si>
-    <t>SAN - SD</t>
-  </si>
-  <si>
-    <t>2026-04-21</t>
-  </si>
-  <si>
-    <t>HK</t>
-  </si>
-  <si>
-    <t>Vahid Balali</t>
-  </si>
-  <si>
-    <t>148686</t>
-  </si>
-  <si>
-    <t>2026-06-01</t>
-  </si>
-  <si>
-    <t>2026-11-01</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69c6e1d59317e8e48f1c9603</t>
-  </si>
-  <si>
-    <t>26-0206</t>
-  </si>
-  <si>
-    <t>Inglewood Transit Connector RFQ</t>
-  </si>
-  <si>
-    <t>Retail</t>
-  </si>
-  <si>
-    <t>2026-03-25</t>
-  </si>
-  <si>
-    <t>2026-04-11</t>
-  </si>
-  <si>
-    <t>Nilda Puno</t>
-  </si>
-  <si>
-    <t>3000</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69c42fb71e34da5627943f29</t>
-  </si>
-  <si>
-    <t>26-0215</t>
-  </si>
-  <si>
-    <t>33P Affordable Housing Multi-Family Devlopment</t>
-  </si>
-  <si>
-    <t>Residential</t>
-  </si>
-  <si>
-    <t>2026-04-15</t>
-  </si>
-  <si>
-    <t>Jon Smith</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69d046a028ff4e0032ca893c</t>
-  </si>
-  <si>
-    <t>26-0216</t>
+    <t>2026-04-17</t>
+  </si>
+  <si>
+    <t>Jonathan Enriquez</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69d403f406964200385d4f8c</t>
+  </si>
+  <si>
+    <t>26-0218</t>
   </si>
   <si>
     <t>GoCary Bus Operations &amp; Maintenance Facility (BOMF)</t>
@@ -353,36 +365,6 @@
   </si>
   <si>
     <t>DeShaun Taylor</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69d3e1fe1fa22b68bef01c78</t>
-  </si>
-  <si>
-    <t>26-0217</t>
-  </si>
-  <si>
-    <t>KR</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69d3de61132a4642c558b4df</t>
-  </si>
-  <si>
-    <t>26-0219</t>
-  </si>
-  <si>
-    <t>Station 33 Bldg 4 Food Hall SD Budget</t>
-  </si>
-  <si>
-    <t>2026-04-17</t>
-  </si>
-  <si>
-    <t>Jonathan Enriquez</t>
-  </si>
-  <si>
-    <t>https://app.buildingconnected.com/opportunities/69d403f406964200385d4f8c</t>
-  </si>
-  <si>
-    <t>26-0218</t>
   </si>
   <si>
     <t>https://app.buildingconnected.com/opportunities/69d3dce067942824a3512727</t>
@@ -784,7 +766,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1069,25 +1051,25 @@
         <v>60</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>61</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="E7" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="F7" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="G7" t="s">
-        <v>17</v>
+        <v>64</v>
       </c>
       <c r="H7" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="I7" t="s">
         <v>17</v>
@@ -1105,18 +1087,18 @@
         <v>17</v>
       </c>
       <c r="N7" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="B8" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C8" t="s">
-        <v>66</v>
+        <v>53</v>
       </c>
       <c r="D8" t="s">
         <v>17</v>
@@ -1125,13 +1107,13 @@
         <v>36</v>
       </c>
       <c r="F8" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G8" t="s">
         <v>17</v>
       </c>
       <c r="H8" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="I8" t="s">
         <v>17</v>
@@ -1149,33 +1131,33 @@
         <v>17</v>
       </c>
       <c r="N8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B9" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C9" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
       <c r="D9" t="s">
-        <v>17</v>
+        <v>75</v>
       </c>
       <c r="E9" t="s">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="F9" t="s">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="G9" t="s">
-        <v>17</v>
+        <v>77</v>
       </c>
       <c r="H9" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="I9" t="s">
         <v>17</v>
@@ -1193,36 +1175,36 @@
         <v>17</v>
       </c>
       <c r="N9" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B10" t="s">
-        <v>76</v>
+        <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>77</v>
+        <v>16</v>
       </c>
       <c r="D10" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="E10" t="s">
-        <v>79</v>
+        <v>18</v>
       </c>
       <c r="F10" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="G10" t="s">
-        <v>17</v>
+        <v>82</v>
       </c>
       <c r="H10" t="s">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="I10" t="s">
-        <v>17</v>
+        <v>83</v>
       </c>
       <c r="J10" t="s">
         <v>58</v>
@@ -1237,127 +1219,127 @@
         <v>17</v>
       </c>
       <c r="N10" t="s">
-        <v>81</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>85</v>
       </c>
       <c r="C11" t="s">
-        <v>16</v>
+        <v>86</v>
       </c>
       <c r="D11" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="E11" t="s">
         <v>18</v>
       </c>
       <c r="F11" t="s">
-        <v>19</v>
+        <v>87</v>
       </c>
       <c r="G11" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="H11" t="s">
-        <v>20</v>
+        <v>89</v>
       </c>
       <c r="I11" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="J11" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="K11" t="s">
-        <v>17</v>
+        <v>91</v>
       </c>
       <c r="L11" t="s">
-        <v>17</v>
+        <v>92</v>
       </c>
       <c r="M11" t="s">
         <v>17</v>
       </c>
       <c r="N11" t="s">
-        <v>23</v>
+        <v>93</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="B12" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="C12" t="s">
-        <v>88</v>
+        <v>16</v>
       </c>
       <c r="D12" t="s">
-        <v>78</v>
+        <v>96</v>
       </c>
       <c r="E12" t="s">
-        <v>18</v>
+        <v>97</v>
       </c>
       <c r="F12" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="G12" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="H12" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="I12" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="J12" t="s">
         <v>40</v>
       </c>
       <c r="K12" t="s">
-        <v>93</v>
+        <v>17</v>
       </c>
       <c r="L12" t="s">
-        <v>94</v>
+        <v>17</v>
       </c>
       <c r="M12" t="s">
         <v>17</v>
       </c>
       <c r="N12" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="B13" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C13" t="s">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="D13" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="E13" t="s">
-        <v>99</v>
+        <v>54</v>
       </c>
       <c r="F13" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="G13" t="s">
-        <v>84</v>
+        <v>17</v>
       </c>
       <c r="H13" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="I13" t="s">
-        <v>102</v>
+        <v>17</v>
       </c>
       <c r="J13" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="K13" t="s">
         <v>17</v>
@@ -1369,33 +1351,33 @@
         <v>17</v>
       </c>
       <c r="N13" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B14" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C14" t="s">
-        <v>26</v>
+        <v>110</v>
       </c>
       <c r="D14" t="s">
-        <v>106</v>
+        <v>75</v>
       </c>
       <c r="E14" t="s">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="F14" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G14" t="s">
-        <v>17</v>
+        <v>82</v>
       </c>
       <c r="H14" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="I14" t="s">
         <v>17</v>
@@ -1413,36 +1395,36 @@
         <v>17</v>
       </c>
       <c r="N14" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B15" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C15" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D15" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E15" t="s">
         <v>37</v>
       </c>
       <c r="F15" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="G15" t="s">
         <v>17</v>
       </c>
       <c r="H15" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="I15" t="s">
-        <v>57</v>
+        <v>17</v>
       </c>
       <c r="J15" t="s">
         <v>58</v>
@@ -1457,143 +1439,11 @@
         <v>17</v>
       </c>
       <c r="N15" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>115</v>
-      </c>
-      <c r="B16" t="s">
-        <v>111</v>
-      </c>
-      <c r="C16" t="s">
-        <v>112</v>
-      </c>
-      <c r="D16" t="s">
-        <v>78</v>
-      </c>
-      <c r="E16" t="s">
-        <v>37</v>
-      </c>
-      <c r="F16" t="s">
-        <v>89</v>
-      </c>
-      <c r="G16" t="s">
-        <v>116</v>
-      </c>
-      <c r="H16" t="s">
-        <v>113</v>
-      </c>
-      <c r="I16" t="s">
-        <v>17</v>
-      </c>
-      <c r="J16" t="s">
-        <v>58</v>
-      </c>
-      <c r="K16" t="s">
-        <v>17</v>
-      </c>
-      <c r="L16" t="s">
-        <v>17</v>
-      </c>
-      <c r="M16" t="s">
-        <v>17</v>
-      </c>
-      <c r="N16" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
         <v>118</v>
-      </c>
-      <c r="B17" t="s">
-        <v>119</v>
-      </c>
-      <c r="C17" t="s">
-        <v>61</v>
-      </c>
-      <c r="D17" t="s">
-        <v>78</v>
-      </c>
-      <c r="E17" t="s">
-        <v>27</v>
-      </c>
-      <c r="F17" t="s">
-        <v>120</v>
-      </c>
-      <c r="G17" t="s">
-        <v>17</v>
-      </c>
-      <c r="H17" t="s">
-        <v>121</v>
-      </c>
-      <c r="I17" t="s">
-        <v>17</v>
-      </c>
-      <c r="J17" t="s">
-        <v>58</v>
-      </c>
-      <c r="K17" t="s">
-        <v>17</v>
-      </c>
-      <c r="L17" t="s">
-        <v>17</v>
-      </c>
-      <c r="M17" t="s">
-        <v>17</v>
-      </c>
-      <c r="N17" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>123</v>
-      </c>
-      <c r="B18" t="s">
-        <v>111</v>
-      </c>
-      <c r="C18" t="s">
-        <v>112</v>
-      </c>
-      <c r="D18" t="s">
-        <v>78</v>
-      </c>
-      <c r="E18" t="s">
-        <v>37</v>
-      </c>
-      <c r="F18" t="s">
-        <v>89</v>
-      </c>
-      <c r="G18" t="s">
-        <v>17</v>
-      </c>
-      <c r="H18" t="s">
-        <v>113</v>
-      </c>
-      <c r="I18" t="s">
-        <v>17</v>
-      </c>
-      <c r="J18" t="s">
-        <v>58</v>
-      </c>
-      <c r="K18" t="s">
-        <v>17</v>
-      </c>
-      <c r="L18" t="s">
-        <v>17</v>
-      </c>
-      <c r="M18" t="s">
-        <v>17</v>
-      </c>
-      <c r="N18" t="s">
-        <v>124</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N18"/>
+  <autoFilter ref="A1:N15"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update the proposal log backup to include all relevant fields
Update the nightly backup process to include all fields from the `proposal_log_entries` table, ensuring a complete data snapshot.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: b8c342de-3a7a-4a8d-b4a3-2df3949c2128
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: aff93941-ff8d-49c6-ad44-7d444636553d
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/f7cd70f1-dedb-4f27-8c85-9633fe48f13e/b8c342de-3a7a-4a8d-b4a3-2df3949c2128/gzyuspu
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/backups/proposal-log-2026-04-09.xlsx
+++ b/backups/proposal-log-2026-04-09.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="130">
   <si>
     <t>Estimate Number</t>
   </si>
@@ -368,6 +368,39 @@
   </si>
   <si>
     <t>https://app.buildingconnected.com/opportunities/69d3dce067942824a3512727</t>
+  </si>
+  <si>
+    <t>26-0220</t>
+  </si>
+  <si>
+    <t>IMA at 200 Market</t>
+  </si>
+  <si>
+    <t>PDX - Idaho</t>
+  </si>
+  <si>
+    <t>2026-04-22</t>
+  </si>
+  <si>
+    <t>Karie Godzik</t>
+  </si>
+  <si>
+    <t>Draft</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69d7cf8f86a4620051a325b4</t>
+  </si>
+  <si>
+    <t>26-0221</t>
+  </si>
+  <si>
+    <t>Blu South Amenity Center</t>
+  </si>
+  <si>
+    <t>Chase Krueger</t>
+  </si>
+  <si>
+    <t>https://app.buildingconnected.com/opportunities/69d6b0da0f694500321aee22</t>
   </si>
 </sst>
 </file>
@@ -766,7 +799,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1442,8 +1475,96 @@
         <v>118</v>
       </c>
     </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>119</v>
+      </c>
+      <c r="B16" t="s">
+        <v>120</v>
+      </c>
+      <c r="C16" t="s">
+        <v>121</v>
+      </c>
+      <c r="D16" t="s">
+        <v>75</v>
+      </c>
+      <c r="E16" t="s">
+        <v>69</v>
+      </c>
+      <c r="F16" t="s">
+        <v>122</v>
+      </c>
+      <c r="G16" t="s">
+        <v>17</v>
+      </c>
+      <c r="H16" t="s">
+        <v>123</v>
+      </c>
+      <c r="I16" t="s">
+        <v>17</v>
+      </c>
+      <c r="J16" t="s">
+        <v>124</v>
+      </c>
+      <c r="K16" t="s">
+        <v>17</v>
+      </c>
+      <c r="L16" t="s">
+        <v>17</v>
+      </c>
+      <c r="M16" t="s">
+        <v>17</v>
+      </c>
+      <c r="N16" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>126</v>
+      </c>
+      <c r="B17" t="s">
+        <v>127</v>
+      </c>
+      <c r="C17" t="s">
+        <v>34</v>
+      </c>
+      <c r="D17" t="s">
+        <v>75</v>
+      </c>
+      <c r="E17" t="s">
+        <v>69</v>
+      </c>
+      <c r="F17" t="s">
+        <v>47</v>
+      </c>
+      <c r="G17" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" t="s">
+        <v>128</v>
+      </c>
+      <c r="I17" t="s">
+        <v>17</v>
+      </c>
+      <c r="J17" t="s">
+        <v>124</v>
+      </c>
+      <c r="K17" t="s">
+        <v>17</v>
+      </c>
+      <c r="L17" t="s">
+        <v>17</v>
+      </c>
+      <c r="M17" t="s">
+        <v>17</v>
+      </c>
+      <c r="N17" t="s">
+        <v>129</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:N15"/>
+  <autoFilter ref="A1:N17"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>